<commit_message>
Add category-based distinct color themes, modal popup for match details, and latest-first date sorting to Match Directory
</commit_message>
<xml_diff>
--- a/public/fcl-matches.xlsx
+++ b/public/fcl-matches.xlsx
@@ -10,6 +10,9 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$1</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -20,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="54">
   <si>
     <t>Date</t>
   </si>
@@ -457,13 +460,121 @@
 🔗 Official Home Post:
 https://www.facebook.com/share/p/18Q4w5CKCx/</t>
   </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>FCL Challenge Cup 2023</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/1FMmHiSBUK/</t>
+  </si>
+  <si>
+    <t>🏆 FCL CHALLENGE CUP 2023 🏆
+♣️ Teams: 08
+♣️ Total Players: 32
+━━━━━━━━━━━━━━━━━━
+📅 TOURNAMENT DETAILS
+━━━━━━━━━━━━━━━━━━
+🗓️ Start Date: 25 January 2023
+🗓️ Closing Date: 10 February 2023
+🏏 Tournament: FCL Challenge Cup 2023
+👥 Participating Teams: 08
+🏐 Total Players: 32
+━━━━━━━━━━━━━━━━━━
+🔗 TOURNAMENT POST
+━━━━━━━━━━━━━━━━━━
+🔗 Match Post: https://www.facebook.com/share/p/1FMmHiSBUK/</t>
+  </si>
+  <si>
+    <t>FCL Friendly Series (Season 20): Brotherhood Series</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/14z1vwPi4Ti/</t>
+  </si>
+  <si>
+    <t>✨ FCL FRIENDLY SERIES — SEASON 20 ✨
+❤️❤️ BROTHERHOOD SERIES ❤️❤️
+━━━━━━━━━━━━━━━━━━
+📅 SERIES DETAILS
+━━━━━━━━━━━━━━━━━━
+🗓️ Start Date: 09 June 2020
+🗓️ End Date: 16 June 2020
+🏏 Series Name: Brotherhood Series
+♻️ Season: 20
+👥 Players Attended: 74
+━━━━━━━━━━━━━━━━━━
+🔗 SERIES POST
+━━━━━━━━━━━━━━━━━━
+🔗 Match Post: https://www.facebook.com/share/p/14z1vwPi4Ti/</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/1FHgEjvzf2/</t>
+  </si>
+  <si>
+    <t>✨ WOW SINGLE MATCH TOURNAMENT ✨
+💞 SEASON 2 — ZONE SQUAD 💞
+━━━━━━━━━━━━━━━━━━
+📅 TOURNAMENT DETAILS
+━━━━━━━━━━━━━━━━━━
+🗓️ Start Date: 20 June 2020
+🗓️ Closing Date: 26 June 2020
+🏏 Tournament Name: WOW Single Match Tournament
+♻️ Season: 2
+👥 Total Players: 64 (Including 4 Managers)
+🗺️ Total Zones: 4
+👥 Groups per Zone: 4
+🏏 Players per Group: 4
+🎯 Qualification: Top 2 players from each group advance to the 2nd Round
+━━━━━━━━━━━━━━━━━━
+🏆 TOURNAMENT FORMAT
+━━━━━━━━━━━━━━━━━━
+🔹 Total Participants: 64
+🔹 Second Round: 32 Players
+🔹 Round of 16: 16 Players
+🔹 Quarter-Finals: 8 Players
+🔹 Semi-Finals: 4 Players
+🔹 Final: 2 Players
+🏆 Champion: 1 Winner
+⚡ Match Format: Direct Knockout from the Second Round
+🎯 Challenge: Luck + Skill
+━━━━━━━━━━━━━━━━━━
+🔗 TOURNAMENT POST
+━━━━━━━━━━━━━━━━━━
+🔗 Match Post: https://www.facebook.com/share/p/1FHgEjvzf2/</t>
+  </si>
+  <si>
+    <t>WOW Single Match Tournament (Season 2)</t>
+  </si>
+  <si>
+    <t>FCL Togetherness Series 2025</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/1ciG63Lmhy/</t>
+  </si>
+  <si>
+    <t>🧿🧿 FCL TOGETHERNESS SERIES 2025 🧿🧿
+🔴 OFFICIAL HOME POST 🔴
+🤝 Unity • Friendship • Brotherhood 🤝
+━━━━━━━━━━━━━━━━━━
+📅 SERIES DETAILS
+━━━━━━━━━━━━━━━━━━
+🗓️ Start Date: 18 September 2025
+🗓️ Closing Date: 02 October 2025
+👥 Total Players: 24
+🏏 Series Name: FCL Togetherness Series 2025
+━━━━━━━━━━━━━━━━━━
+🔗 SERIES POST
+━━━━━━━━━━━━━━━━━━
+🔗 Match Post: https://www.facebook.com/share/p/1ciG63Lmhy/</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -514,17 +625,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -820,7 +931,7 @@
     <col min="2" max="2" width="9.140625" style="1"/>
     <col min="3" max="3" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="55.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
     <col min="7" max="7" width="49.140625" style="3" bestFit="1" customWidth="1"/>
   </cols>
@@ -1056,40 +1167,96 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="10"/>
+      <c r="A11" s="6">
+        <v>44951</v>
+      </c>
+      <c r="B11" s="7">
+        <v>2023</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="10"/>
+      <c r="A12" s="6">
+        <v>43991</v>
+      </c>
+      <c r="B12" s="7">
+        <v>2020</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="10"/>
+      <c r="A13" s="6">
+        <v>44002</v>
+      </c>
+      <c r="B13" s="7">
+        <v>2020</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="10"/>
+      <c r="A14" s="6">
+        <v>45918</v>
+      </c>
+      <c r="B14" s="7">
+        <v>2025</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
@@ -1290,6 +1457,7 @@
       <c r="G36" s="10"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Player Directory layout with icon grid buttons and fix player card birthday format
</commit_message>
<xml_diff>
--- a/public/fcl-matches.xlsx
+++ b/public/fcl-matches.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$1</definedName>
@@ -23,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="66">
   <si>
     <t>Date</t>
   </si>
@@ -568,6 +567,214 @@
 ━━━━━━━━━━━━━━━━━━
 🔗 Match Post: https://www.facebook.com/share/p/1ciG63Lmhy/</t>
   </si>
+  <si>
+    <t>Official Friendly Match: FCL Godzillas vs FCL Kingkongs</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/1J1ExCu3PX/</t>
+  </si>
+  <si>
+    <t>✨ FCL OFFICIAL FRIENDLY MATCH ✨
+♦️ FCL GODZILLAS 🆚 FCL KINGKONGS ♦️
+━━━━━━━━━━━━━━━━━━
+📅 MATCH DETAILS
+━━━━━━━━━━━━━━━━━━
+🗓️ Date: 15 October 2026
+⏰ Start Time: 09:17 PM
+🏁 Closing Time: 10:07 PM
+⏱️ Duration: 51 minutes
+🏟️ Venue: FCL National Cricket Ground
+♻️ Format: T20+
+🏐 Match Type: 5 Overs &amp; 7 Wickets
+🏏 Powerplay: 2nd Over Bowling Powerplay &amp; 4th Over Batting Powerplay
+━━━━━━━━━━━━━━━━━━
+⚡ FCL GODZILLAS SQUAD
+━━━━━━━━━━━━━━━━━━
+1. Asif Iqbal Khan (C)
+2. Shahriar Khan Shovon
+3. Rakibul Islam (VC)
+4. Tanvir Shakib
+━━━━━━━━━━━━━━━━━━
+⚡ FCL KINGKONGS SQUAD
+━━━━━━━━━━━━━━━━━━
+1. Md Ridoy AR
+2. Susmoy Paul (C)
+3. M R Shakil (VC)
+4. Md Siyam Islam
+━━━━━━━━━━━━━━━━━━
+🏏 MATCH SUMMARY
+━━━━━━━━━━━━━━━━━━
+🪙 Toss: FCL Godzillas won the toss and chose to bowl first.
+🔹 FCL Kingkongs: 67/7 (4.4 Overs)
+🎯 Target: 68 Runs
+🔹 FCL Godzillas: 69/4 (4.0 Overs)
+🏆 Result: FCL Godzillas won by 3 wickets!
+━━━━━━━━━━━━━━━━━━
+🏅 INDIVIDUAL AWARDS
+━━━━━━━━━━━━━━━━━━
+🌟 Man of the Match (MOM): Tanvir Shakib — 353 Impact Points
+💎 Chief Player of the Match (CPOM): Susmoy Paul — 251 Impact Points</t>
+  </si>
+  <si>
+    <t>Birthday Special Friendly Match: Adnan Warriors vs Akash Titans</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/19beZuLYzi/</t>
+  </si>
+  <si>
+    <t>✨ FCL BIRTHDAY SPECIAL FRIENDLY MATCH ✨
+♦️ ADNAN WARRIORS 🆚 AKASH TITANS ♦️
+━━━━━━━━━━━━━━━━━━
+📅 MATCH DETAILS
+━━━━━━━━━━━━━━━━━━
+🗓️ Date: 16 October 2026
+⏰ Start Time: 09:22 PM
+🏁 Closing Time: 10:09 PM
+⏱️ Duration: 47 minutes
+🏟️ Venue: FCL National Cricket Ground
+♻️ Format: T20+
+🏐 Match Type: 5 Overs &amp; 7 Wickets
+🏏 Powerplay: 2nd Over Bowling Powerplay &amp; 4th Over Batting Powerplay
+━━━━━━━━━━━━━━━━━━
+⚡ ADNAN WARRIORS SQUAD
+━━━━━━━━━━━━━━━━━━
+1. Susmoy Paul (C)
+2. M R Shakil (VC)
+3. Md Ridoy AR
+4. Shah Abi Talib Adnan
+5. Nur Muhammad
+━━━━━━━━━━━━━━━━━━
+⚡ AKASH TITANS SQUAD
+━━━━━━━━━━━━━━━━━━
+1. Asif Iqbal Khan (C)
+2. Mahabubur Rahman Akásh
+3. Shahriar Khan Shovon
+4. Md Siyam Islam
+5. Rakibul Islam (VC)
+━━━━━━━━━━━━━━━━━━
+🏏 MATCH SUMMARY
+━━━━━━━━━━━━━━━━━━
+🪙 Toss: Akash Titans won the toss and chose to bowl first.
+🔹 Adnan Warriors: 88/4 (5.0 Overs)
+🎯 Target: 89 Runs
+🔹 Akash Titans: 31/7 (2.3 Overs)
+🏆 Result: Adnan Warriors won by 57 runs!
+━━━━━━━━━━━━━━━━━━
+🏅 INDIVIDUAL AWARDS
+━━━━━━━━━━━━━━━━━━
+🌟 Man of the Match (MOM): AM Adnan vai — 279 Impact Points
+💎 Chief Player of the Match (CPOM): M R Shakil — 264 Impact Points
+━━━━━━━━━━━━━━━━━━
+🔗 MATCH POST
+━━━━━━━━━━━━━━━━━━
+🔗 Match Post: https://www.facebook.com/share/p/19beZuLYzi/</t>
+  </si>
+  <si>
+    <t>Special Friendly Match: FCL Superstars vs FCL Underdogs</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/1FT3P7VQ5Q/</t>
+  </si>
+  <si>
+    <t>✨ FCL SPECIAL FRIENDLY MATCH ✨
+♦️ FCL SUPERSTARS 🆚 FCL UNDERDOGS ♦️
+━━━━━━━━━━━━━━━━━━
+📅 MATCH DETAILS
+━━━━━━━━━━━━━━━━━━
+🗓️ Date: 17 October 2026
+⏰ Start Time: 09:33 PM
+🏁 Closing Time: 10:37 PM
+⏱️ Duration: 64 minutes
+🏟️ Venue: FCL National Cricket Ground
+♻️ Format: T20+
+🏐 Match Type: 5 Overs &amp; 7 Wickets
+🏏 Powerplay: 2nd Over Bowling Powerplay &amp; 4th Over Batting Powerplay
+━━━━━━━━━━━━━━━━━━
+⚡ FCL SUPERSTARS SQUAD
+━━━━━━━━━━━━━━━━━━
+1. Asif Iqbal Khan
+2. Md Ridoy AR
+3. M R Shakil (VC)
+4. Susmoy Paul (C)
+5. Md Siyam Islam
+━━━━━━━━━━━━━━━━━━
+⚡ FCL UNDERDOGS SQUAD
+━━━━━━━━━━━━━━━━━━
+1. Shahriar Khan Shovon (VC)
+2. Rakibul Islam (C)
+3. আরিফ জিয়াদ
+4. Sayed Anwar Shanto
+5. Sadrul Anam
+━━━━━━━━━━━━━━━━━━
+🏏 MATCH SUMMARY
+━━━━━━━━━━━━━━━━━━
+🪙 Toss: FCL Underdogs won the toss and chose to bowl first.
+🔹 FCL Superstars: 90/5 (5.0 Overs)
+🎯 Target: 91 Runs
+🔹 FCL Underdogs: 48/7 (3.4 Overs)
+🏆 Result: FCL Superstars won by 42 runs!
+━━━━━━━━━━━━━━━━━━
+🏅 INDIVIDUAL AWARDS
+━━━━━━━━━━━━━━━━━━
+🌟 Man of the Match (MOM): Susmoy Paul — 308 Impact Points
+💎 Chief Player of the Match (CPOM): M R Shakil — 232 Impact Points
+━━━━━━━━━━━━━━━━━━
+🔗 MATCH POST
+━━━━━━━━━━━━━━━━━━
+🔗 Match Post: https://www.facebook.com/share/p/1FT3P7VQ5Q/</t>
+  </si>
+  <si>
+    <t>Birthday Special Match: SH Gladiators vs Rubel Burners</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/share/p/1Edr9PSdcM/</t>
+  </si>
+  <si>
+    <t>✨ FCL BIRTHDAY SPECIAL FRIENDLY MATCH ✨
+♦️ SH GLADIATORS 🆚 RUBEL BURNERS ♦️
+━━━━━━━━━━━━━━━━━━
+📅 MATCH DETAILS
+━━━━━━━━━━━━━━━━━━
+🗓️ Date: 17 October 2026
+⏰ Start Time: 09:40 PM
+🏁 Closing Time: 10:29 PM
+⏱️ Duration: 49 minutes
+🏟️ Venue: FCL National Cricket Ground
+♻️ Format: T20+
+🏐 Match Type: 5 Overs &amp; 7 Wickets
+🏏 Powerplay: 2nd Over Bowling Powerplay &amp; 4th Over Batting Powerplay
+━━━━━━━━━━━━━━━━━━
+⚡ SH GLADIATORS SQUAD
+━━━━━━━━━━━━━━━━━━
+1. Kamil Ahmed
+2. MD Tofayel Ahmed (C)
+3. Sakhawat Hossain Shanto (VC)
+4. Zaheed Hasan
+━━━━━━━━━━━━━━━━━━
+⚡ RUBEL BURNERS SQUAD
+━━━━━━━━━━━━━━━━━━
+1. মোঃ আশিকুর রহমান তন্ময় (C)
+2. ShiShir Hossain
+3. Prince Tarek
+4. Raian Jabir (VC)
+━━━━━━━━━━━━━━━━━━
+🏏 MATCH SUMMARY
+━━━━━━━━━━━━━━━━━━
+🪙 Toss: SH Gladiators won the toss and chose to bowl first.
+🔹 Rubel Burners: 99/4 (5.0 Overs)
+🎯 Target: 100 Runs
+🔹 SH Gladiators: 87/5 (5.0 Overs)
+🏆 Result: Rubel Burners won by 12 runs!
+━━━━━━━━━━━━━━━━━━
+🏅 INDIVIDUAL AWARDS
+━━━━━━━━━━━━━━━━━━
+🌟 Man of the Match (MOM): Prince Tarek — 294 Impact Points
+💎 Chief Player of the Match (CPOM): Zaheed Hasan — 287 Impact Points
+━━━━━━━━━━━━━━━━━━
+🔗 MATCH POST
+━━━━━━━━━━━━━━━━━━
+🔗 Match Post: https://www.facebook.com/share/p/1Edr9PSdcM/</t>
+  </si>
 </sst>
 </file>
 
@@ -576,10 +783,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -617,10 +832,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -644,8 +860,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -929,7 +1149,7 @@
   <cols>
     <col min="1" max="1" width="12.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.140625" style="1"/>
-    <col min="3" max="3" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="55.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
@@ -1259,40 +1479,96 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="10"/>
+      <c r="A15" s="6">
+        <v>46310</v>
+      </c>
+      <c r="B15" s="7">
+        <v>2026</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="6"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="10"/>
+      <c r="A16" s="6">
+        <v>46311</v>
+      </c>
+      <c r="B16" s="7">
+        <v>2026</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="10"/>
+      <c r="A17" s="6">
+        <v>46312</v>
+      </c>
+      <c r="B17" s="7">
+        <v>2026</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="10"/>
+      <c r="A18" s="6">
+        <v>46312</v>
+      </c>
+      <c r="B18" s="7">
+        <v>2026</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
@@ -1458,16 +1734,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
+  <hyperlinks>
+    <hyperlink ref="G15" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>